<commit_message>
Sorted blog category pages ascending.
</commit_message>
<xml_diff>
--- a/migration/page_list.xlsx
+++ b/migration/page_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick/dev/Elseyworld/migration/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{FF166B8B-7474-964B-99D0-D4503FEEA019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1180B256-5E4D-EF48-9A6D-EC4590D0C822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="53900" yWindow="620" windowWidth="22900" windowHeight="41300" xr2:uid="{E1FA346A-4A23-AB4F-9BF3-1F63A6AB369D}"/>
   </bookViews>
@@ -1293,11 +1293,17 @@
       <c r="A10" t="s">
         <v>24</v>
       </c>
+      <c r="B10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>20</v>
       </c>
+      <c r="B11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -1746,6 +1752,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Reviewed all Lynn articles
</commit_message>
<xml_diff>
--- a/migration/page_list.xlsx
+++ b/migration/page_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick/dev/Elseyworld/migration/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1180B256-5E4D-EF48-9A6D-EC4590D0C822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52BC9629-D43F-3448-AB9B-281CD104B460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="53900" yWindow="620" windowWidth="22900" windowHeight="41300" xr2:uid="{E1FA346A-4A23-AB4F-9BF3-1F63A6AB369D}"/>
   </bookViews>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">page_list!$A$2:$A$100</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1309,25 +1322,40 @@
       <c r="A12" t="s">
         <v>5</v>
       </c>
+      <c r="B12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>3</v>
       </c>
+      <c r="B13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>4</v>
       </c>
+      <c r="B14" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>0</v>
       </c>
+      <c r="B15" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>6</v>
+      </c>
+      <c r="B16" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Australia trip 2 cleanup
</commit_message>
<xml_diff>
--- a/migration/page_list.xlsx
+++ b/migration/page_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick/dev/Elseyworld/migration/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{577187D3-A687-CD41-8E54-F7F43392BA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{466BD114-8544-9F45-861E-F745D5B18157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="53900" yWindow="620" windowWidth="22900" windowHeight="41300" xr2:uid="{E1FA346A-4A23-AB4F-9BF3-1F63A6AB369D}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="page_list" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">page_list!$A$2:$A$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">page_list!$A$2:$A$87</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
   <si>
     <t>articles/food-travel/salishan</t>
   </si>
@@ -294,45 +294,6 @@
   </si>
   <si>
     <t>blog/asia-2009/hoa-binh-or-bust</t>
-  </si>
-  <si>
-    <t>categories/food-travel</t>
-  </si>
-  <si>
-    <t>categories/nick</t>
-  </si>
-  <si>
-    <t>categories/magazines</t>
-  </si>
-  <si>
-    <t>categories/health</t>
-  </si>
-  <si>
-    <t>categories/business</t>
-  </si>
-  <si>
-    <t>categories/australia-2002-trip-2</t>
-  </si>
-  <si>
-    <t>categories/careers</t>
-  </si>
-  <si>
-    <t>categories/south-pacific-1997</t>
-  </si>
-  <si>
-    <t>categories/moving-to-dc</t>
-  </si>
-  <si>
-    <t>categories/lynn</t>
-  </si>
-  <si>
-    <t>categories/australia-2009</t>
-  </si>
-  <si>
-    <t>categories/australia-2002-trip-1</t>
-  </si>
-  <si>
-    <t>categories/asia-2009</t>
   </si>
   <si>
     <t>Folder</t>
@@ -889,10 +850,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EF049980-CE74-4140-80AF-C610CEAB5092}" name="Table1" displayName="Table1" ref="A1:C100" totalsRowShown="0">
-  <autoFilter ref="A1:C100" xr:uid="{EF049980-CE74-4140-80AF-C610CEAB5092}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C100">
-    <sortCondition ref="A1:A100"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EF049980-CE74-4140-80AF-C610CEAB5092}" name="Table1" displayName="Table1" ref="A1:C87" totalsRowShown="0">
+  <autoFilter ref="A1:C87" xr:uid="{EF049980-CE74-4140-80AF-C610CEAB5092}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C87">
+    <sortCondition ref="A1:A87"/>
   </sortState>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{FFE08CDC-8687-E143-9074-104FBFEB18A7}" name="Folder"/>
@@ -1220,7 +1181,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B86FC75E-37C9-1C4F-8B68-98E9A071B500}">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="68.6640625" bestFit="1" customWidth="1"/>
@@ -1229,13 +1190,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="B1" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="C1" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -1299,7 +1260,7 @@
         <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -1594,93 +1555,117 @@
       <c r="A46" t="s">
         <v>64</v>
       </c>
+      <c r="B46" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>61</v>
       </c>
+      <c r="B47" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B52" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>59</v>
       </c>
@@ -1798,71 +1783,6 @@
     <row r="87" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
-        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Australia 2009, 2002 trip 2
</commit_message>
<xml_diff>
--- a/migration/page_list.xlsx
+++ b/migration/page_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick/dev/Elseyworld/migration/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{466BD114-8544-9F45-861E-F745D5B18157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE3B39D4-EEE0-E343-AE9D-640161DE0111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="53900" yWindow="620" windowWidth="22900" windowHeight="41300" xr2:uid="{E1FA346A-4A23-AB4F-9BF3-1F63A6AB369D}"/>
   </bookViews>
@@ -851,7 +851,11 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EF049980-CE74-4140-80AF-C610CEAB5092}" name="Table1" displayName="Table1" ref="A1:C87" totalsRowShown="0">
-  <autoFilter ref="A1:C87" xr:uid="{EF049980-CE74-4140-80AF-C610CEAB5092}"/>
+  <autoFilter ref="A1:C87" xr:uid="{EF049980-CE74-4140-80AF-C610CEAB5092}">
+    <filterColumn colId="1">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C87">
     <sortCondition ref="A1:A87"/>
   </sortState>
@@ -1199,7 +1203,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1207,7 +1211,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -1215,7 +1219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1223,7 +1227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1231,7 +1235,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -1239,7 +1243,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -1247,7 +1251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1255,7 +1259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1263,7 +1267,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1271,7 +1275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1279,7 +1283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -1287,7 +1291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1295,7 +1299,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1303,7 +1307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -1311,7 +1315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -1319,7 +1323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -1327,7 +1331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>1</v>
       </c>
@@ -1335,7 +1339,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -1343,7 +1347,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>13</v>
       </c>
@@ -1351,7 +1355,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -1359,7 +1363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>10</v>
       </c>
@@ -1367,7 +1371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>11</v>
       </c>
@@ -1375,7 +1379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -1383,7 +1387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -1391,7 +1395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>7</v>
       </c>
@@ -1399,7 +1403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -1407,7 +1411,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>68</v>
       </c>
@@ -1415,7 +1419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>70</v>
       </c>
@@ -1423,7 +1427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>76</v>
       </c>
@@ -1431,7 +1435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>72</v>
       </c>
@@ -1439,7 +1443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>84</v>
       </c>
@@ -1447,7 +1451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>71</v>
       </c>
@@ -1455,7 +1459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>77</v>
       </c>
@@ -1463,7 +1467,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>78</v>
       </c>
@@ -1471,7 +1475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>75</v>
       </c>
@@ -1479,7 +1483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>74</v>
       </c>
@@ -1487,7 +1491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>85</v>
       </c>
@@ -1495,7 +1499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>69</v>
       </c>
@@ -1503,7 +1507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>73</v>
       </c>
@@ -1511,7 +1515,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>79</v>
       </c>
@@ -1519,7 +1523,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>83</v>
       </c>
@@ -1527,7 +1531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>81</v>
       </c>
@@ -1535,7 +1539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>82</v>
       </c>
@@ -1543,7 +1547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>80</v>
       </c>
@@ -1551,7 +1555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>64</v>
       </c>
@@ -1559,7 +1563,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>61</v>
       </c>
@@ -1567,7 +1571,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>67</v>
       </c>
@@ -1575,7 +1579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>60</v>
       </c>
@@ -1583,7 +1587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>62</v>
       </c>
@@ -1591,7 +1595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>63</v>
       </c>
@@ -1599,7 +1603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>66</v>
       </c>
@@ -1607,7 +1611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>65</v>
       </c>
@@ -1619,133 +1623,187 @@
       <c r="A54" t="s">
         <v>27</v>
       </c>
+      <c r="B54" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>26</v>
       </c>
+      <c r="B55" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>29</v>
       </c>
+      <c r="B56" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>28</v>
       </c>
+      <c r="B57" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>46</v>
       </c>
+      <c r="B58" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>50</v>
       </c>
+      <c r="B59" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>58</v>
       </c>
+      <c r="B60" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>57</v>
       </c>
+      <c r="B61" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>47</v>
       </c>
+      <c r="B62" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>48</v>
       </c>
+      <c r="B63" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B64" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B65" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B66" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B67" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B68" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B69" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B70" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B71" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>33</v>
       </c>

</xml_diff>